<commit_message>
Fix subida campaña excel
</commit_message>
<xml_diff>
--- a/Formatos/Formato Ficha QP.xlsx
+++ b/Formatos/Formato Ficha QP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Python\Proyecto Control QP\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F091D9A-DC93-4B42-B49A-9FE1DEC417C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E880B7A6-5DA5-4D0F-9082-4AB137D4A2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2FFCEFF2-5F86-44FA-BEF3-06B9FA732BBA}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
   <si>
     <t>CODIGO CAMPAÑA:</t>
   </si>
@@ -51,15 +51,6 @@
     <t>FECHA FIN:</t>
   </si>
   <si>
-    <t>QP-QUA-002</t>
-  </si>
-  <si>
-    <t>QUASAR02</t>
-  </si>
-  <si>
-    <t>QUASAR</t>
-  </si>
-  <si>
     <t>TIENDAS</t>
   </si>
   <si>
@@ -78,91 +69,88 @@
     <t>Provincia</t>
   </si>
   <si>
-    <t>Tienda1</t>
-  </si>
-  <si>
-    <t>Tienda2</t>
-  </si>
-  <si>
-    <t>Tienda3</t>
-  </si>
-  <si>
-    <t>Tienda4</t>
-  </si>
-  <si>
-    <t>Tienda5</t>
-  </si>
-  <si>
-    <t>Tienda6</t>
-  </si>
-  <si>
-    <t>Tienda7</t>
-  </si>
-  <si>
-    <t>Tienda8</t>
-  </si>
-  <si>
-    <t>Tienda9</t>
-  </si>
-  <si>
-    <t>Tienda10</t>
-  </si>
-  <si>
     <t>Lima</t>
   </si>
   <si>
-    <t>Producto1</t>
-  </si>
-  <si>
-    <t>Producto2</t>
-  </si>
-  <si>
-    <t>Producto3</t>
-  </si>
-  <si>
-    <t>Producto4</t>
-  </si>
-  <si>
-    <t>Producto5</t>
-  </si>
-  <si>
-    <t>Producto6</t>
-  </si>
-  <si>
-    <t>Producto7</t>
-  </si>
-  <si>
-    <t>Producto8</t>
-  </si>
-  <si>
-    <t>Producto9</t>
-  </si>
-  <si>
-    <t>Producto10</t>
-  </si>
-  <si>
     <t>Unidad</t>
   </si>
   <si>
-    <t>Caja</t>
-  </si>
-  <si>
     <t>Paquete</t>
   </si>
   <si>
-    <t>Six Pack</t>
-  </si>
-  <si>
     <t>Uniformes</t>
   </si>
   <si>
-    <t>Merchandising</t>
-  </si>
-  <si>
     <t>Insumos</t>
   </si>
   <si>
     <t>Perecibles</t>
+  </si>
+  <si>
+    <t>QP-AJE-0001</t>
+  </si>
+  <si>
+    <t>AJE</t>
+  </si>
+  <si>
+    <t>HEY FIT</t>
+  </si>
+  <si>
+    <t>PVEA SALAVERRY</t>
+  </si>
+  <si>
+    <t>PVEA SUCRE</t>
+  </si>
+  <si>
+    <t>PVEA CALLAO</t>
+  </si>
+  <si>
+    <t>PVEA MIRAFLORES</t>
+  </si>
+  <si>
+    <t>PVEA SAN BORJA</t>
+  </si>
+  <si>
+    <t>PVEA AREQUIPA</t>
+  </si>
+  <si>
+    <t>PVEA TRUJILLO</t>
+  </si>
+  <si>
+    <t>PVEA CHICLAYO</t>
+  </si>
+  <si>
+    <t>PVEA PIURA</t>
+  </si>
+  <si>
+    <t>PVEA CHIMBOTE</t>
+  </si>
+  <si>
+    <t>HEY FIT TORONJA</t>
+  </si>
+  <si>
+    <t>HEY FIT PIÑA</t>
+  </si>
+  <si>
+    <t>HEY FIT GOLDEN</t>
+  </si>
+  <si>
+    <t>COOLER ROJO</t>
+  </si>
+  <si>
+    <t>VASOS 5 OZ</t>
+  </si>
+  <si>
+    <t>POLO</t>
+  </si>
+  <si>
+    <t>FALDA</t>
+  </si>
+  <si>
+    <t>GORRA</t>
+  </si>
+  <si>
+    <t>Elementos</t>
   </si>
 </sst>
 </file>
@@ -743,20 +731,20 @@
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="D4" s="5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -764,22 +752,22 @@
         <v>0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="I5" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -787,22 +775,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H6" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="I6" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -810,22 +798,22 @@
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" t="s">
         <v>16</v>
-      </c>
-      <c r="E7" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -833,22 +821,22 @@
         <v>3</v>
       </c>
       <c r="B8" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="H8" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="I8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -856,107 +844,89 @@
         <v>4</v>
       </c>
       <c r="B9" s="3">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G9" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="H9" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="I9" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H10" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="I10" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D11" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" t="s">
         <v>13</v>
       </c>
-      <c r="G11" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" t="s">
-        <v>37</v>
-      </c>
       <c r="I11" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="E12" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H12" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="I12" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D13" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" t="s">
-        <v>38</v>
-      </c>
-      <c r="I13" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D14" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" t="s">
-        <v>34</v>
-      </c>
-      <c r="H14" t="s">
-        <v>38</v>
-      </c>
-      <c r="I14" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>